<commit_message>
Comentarios y predicctor en funcionamiento con prevision de ventas
</commit_message>
<xml_diff>
--- a/data/inputs/horarios.xlsx
+++ b/data/inputs/horarios.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jaimeteran/Documents/PYTHON/vacanze_romane/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jaimeteran/Documents/PYTHON/VacanzeGIT/data/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{654E0D37-890D-2142-B76C-A6F6E5C21B84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E66ACBB-4184-7447-8BA0-666FD35A21E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17160" xr2:uid="{12839FEE-75C8-E040-B05A-1C8EEF2279EC}"/>
   </bookViews>

</xml_diff>